<commit_message>
sebelum penghapusan heuristik octile
</commit_message>
<xml_diff>
--- a/Excel/Vertical/hasil_gabungan_semua_sheet.xlsx
+++ b/Excel/Vertical/hasil_gabungan_semua_sheet.xlsx
@@ -477,7 +477,7 @@
         <v>16</v>
       </c>
       <c r="C2">
-        <v>0.0004822</v>
+        <v>0.0005032000000000001</v>
       </c>
       <c r="D2" t="s">
         <v>3</v>
@@ -509,7 +509,7 @@
         <v>16</v>
       </c>
       <c r="C3">
-        <v>0.0002534999999999999</v>
+        <v>0.0002433</v>
       </c>
       <c r="D3" t="s">
         <v>3</v>
@@ -541,7 +541,7 @@
         <v>16</v>
       </c>
       <c r="C4">
-        <v>0.0004101</v>
+        <v>0.0001963</v>
       </c>
       <c r="D4" t="s">
         <v>3</v>
@@ -573,7 +573,7 @@
         <v>16</v>
       </c>
       <c r="C5">
-        <v>0.0003179</v>
+        <v>0.0003287</v>
       </c>
       <c r="D5" t="s">
         <v>3</v>
@@ -605,7 +605,7 @@
         <v>16</v>
       </c>
       <c r="C6">
-        <v>0.0003319</v>
+        <v>0.0003375</v>
       </c>
       <c r="D6" t="s">
         <v>3</v>
@@ -637,16 +637,16 @@
         <v>16</v>
       </c>
       <c r="C7">
-        <v>0.0005113</v>
+        <v>0.0004804</v>
       </c>
       <c r="D7" t="s">
         <v>3</v>
       </c>
       <c r="E7">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F7">
-        <v>23.09901951359279</v>
+        <v>23.12310562561766</v>
       </c>
       <c r="G7">
         <v>30</v>
@@ -655,7 +655,7 @@
         <v>58</v>
       </c>
       <c r="I7">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J7">
         <v>88</v>
@@ -669,7 +669,7 @@
         <v>16</v>
       </c>
       <c r="C8">
-        <v>0.0005372</v>
+        <v>0.0005020000000000001</v>
       </c>
       <c r="D8" t="s">
         <v>3</v>
@@ -681,16 +681,16 @@
         <v>24.14213562373095</v>
       </c>
       <c r="G8">
-        <v>32</v>
+        <v>38</v>
       </c>
       <c r="H8">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="I8">
         <v>9</v>
       </c>
       <c r="J8">
-        <v>91</v>
+        <v>96</v>
       </c>
     </row>
     <row r="9" spans="1:10">
@@ -701,7 +701,7 @@
         <v>32</v>
       </c>
       <c r="C9">
-        <v>0.0034743</v>
+        <v>0.003523399999999999</v>
       </c>
       <c r="D9" t="s">
         <v>3</v>
@@ -733,7 +733,7 @@
         <v>32</v>
       </c>
       <c r="C10">
-        <v>0.0011258</v>
+        <v>0.0011045</v>
       </c>
       <c r="D10" t="s">
         <v>3</v>
@@ -765,7 +765,7 @@
         <v>32</v>
       </c>
       <c r="C11">
-        <v>0.0013158</v>
+        <v>0.0006369999999999999</v>
       </c>
       <c r="D11" t="s">
         <v>3</v>
@@ -780,13 +780,13 @@
         <v>103</v>
       </c>
       <c r="H11">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="I11">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="J11">
-        <v>148</v>
+        <v>145</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -797,7 +797,7 @@
         <v>32</v>
       </c>
       <c r="C12">
-        <v>0.0018366</v>
+        <v>0.0018679</v>
       </c>
       <c r="D12" t="s">
         <v>3</v>
@@ -829,7 +829,7 @@
         <v>32</v>
       </c>
       <c r="C13">
-        <v>0.0010794</v>
+        <v>0.0011568</v>
       </c>
       <c r="D13" t="s">
         <v>3</v>
@@ -861,16 +861,16 @@
         <v>32</v>
       </c>
       <c r="C14">
-        <v>0.0035126</v>
+        <v>0.0034676</v>
       </c>
       <c r="D14" t="s">
         <v>3</v>
       </c>
       <c r="E14">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F14">
-        <v>46.86645192953345</v>
+        <v>47.00870142385959</v>
       </c>
       <c r="G14">
         <v>76</v>
@@ -879,7 +879,7 @@
         <v>241</v>
       </c>
       <c r="I14">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J14">
         <v>317</v>
@@ -893,7 +893,7 @@
         <v>32</v>
       </c>
       <c r="C15">
-        <v>0.003432800000000001</v>
+        <v>0.0033985</v>
       </c>
       <c r="D15" t="s">
         <v>3</v>
@@ -905,7 +905,7 @@
         <v>49.698484809835</v>
       </c>
       <c r="G15">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="H15">
         <v>250</v>
@@ -914,7 +914,7 @@
         <v>10</v>
       </c>
       <c r="J15">
-        <v>316</v>
+        <v>320</v>
       </c>
     </row>
     <row r="16" spans="1:10">
@@ -925,7 +925,7 @@
         <v>64</v>
       </c>
       <c r="C16">
-        <v>0.025808</v>
+        <v>0.0245314</v>
       </c>
       <c r="D16" t="s">
         <v>3</v>
@@ -957,7 +957,7 @@
         <v>64</v>
       </c>
       <c r="C17">
-        <v>0.004922699999999999</v>
+        <v>0.004874399999999999</v>
       </c>
       <c r="D17" t="s">
         <v>3</v>
@@ -989,7 +989,7 @@
         <v>64</v>
       </c>
       <c r="C18">
-        <v>0.005923699999999999</v>
+        <v>0.0020404</v>
       </c>
       <c r="D18" t="s">
         <v>3</v>
@@ -998,19 +998,19 @@
         <v>84</v>
       </c>
       <c r="F18">
-        <v>103.2964645562817</v>
+        <v>102.4680374315355</v>
       </c>
       <c r="G18">
-        <v>264</v>
+        <v>219</v>
       </c>
       <c r="H18">
-        <v>142</v>
+        <v>88</v>
       </c>
       <c r="I18">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="J18">
-        <v>406</v>
+        <v>307</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -1021,7 +1021,7 @@
         <v>64</v>
       </c>
       <c r="C19">
-        <v>0.0129962</v>
+        <v>0.0127819</v>
       </c>
       <c r="D19" t="s">
         <v>3</v>
@@ -1053,7 +1053,7 @@
         <v>64</v>
       </c>
       <c r="C20">
-        <v>0.0036981</v>
+        <v>0.0036926</v>
       </c>
       <c r="D20" t="s">
         <v>3</v>
@@ -1085,7 +1085,7 @@
         <v>64</v>
       </c>
       <c r="C21">
-        <v>0.0248513</v>
+        <v>0.0243821</v>
       </c>
       <c r="D21" t="s">
         <v>3</v>
@@ -1094,7 +1094,7 @@
         <v>7</v>
       </c>
       <c r="F21">
-        <v>95.40233038888984</v>
+        <v>95.48180327461259</v>
       </c>
       <c r="G21">
         <v>166</v>
@@ -1117,7 +1117,7 @@
         <v>64</v>
       </c>
       <c r="C22">
-        <v>0.0224448</v>
+        <v>0.0220048</v>
       </c>
       <c r="D22" t="s">
         <v>3</v>
@@ -1129,7 +1129,7 @@
         <v>100.8111831820431</v>
       </c>
       <c r="G22">
-        <v>159</v>
+        <v>166</v>
       </c>
       <c r="H22">
         <v>1005</v>
@@ -1138,7 +1138,7 @@
         <v>12</v>
       </c>
       <c r="J22">
-        <v>1164</v>
+        <v>1171</v>
       </c>
     </row>
     <row r="23" spans="1:10">
@@ -1149,7 +1149,7 @@
         <v>128</v>
       </c>
       <c r="C23">
-        <v>0.15967</v>
+        <v>0.1620138</v>
       </c>
       <c r="D23" t="s">
         <v>3</v>
@@ -1181,7 +1181,7 @@
         <v>128</v>
       </c>
       <c r="C24">
-        <v>0.0205536</v>
+        <v>0.0203735</v>
       </c>
       <c r="D24" t="s">
         <v>3</v>
@@ -1213,7 +1213,7 @@
         <v>128</v>
       </c>
       <c r="C25">
-        <v>0.0429991</v>
+        <v>0.0074792</v>
       </c>
       <c r="D25" t="s">
         <v>3</v>
@@ -1222,19 +1222,19 @@
         <v>168</v>
       </c>
       <c r="F25">
-        <v>208.0071426749365</v>
+        <v>206.350288425444</v>
       </c>
       <c r="G25">
-        <v>643</v>
+        <v>460</v>
       </c>
       <c r="H25">
-        <v>587</v>
+        <v>196</v>
       </c>
       <c r="I25">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="J25">
-        <v>1230</v>
+        <v>656</v>
       </c>
     </row>
     <row r="26" spans="1:10">
@@ -1245,7 +1245,7 @@
         <v>128</v>
       </c>
       <c r="C26">
-        <v>0.08562030000000001</v>
+        <v>0.08665039999999999</v>
       </c>
       <c r="D26" t="s">
         <v>3</v>
@@ -1277,7 +1277,7 @@
         <v>128</v>
       </c>
       <c r="C27">
-        <v>0.0150779</v>
+        <v>0.015071</v>
       </c>
       <c r="D27" t="s">
         <v>3</v>
@@ -1309,7 +1309,7 @@
         <v>128</v>
       </c>
       <c r="C28">
-        <v>0.1598635</v>
+        <v>0.1615691</v>
       </c>
       <c r="D28" t="s">
         <v>3</v>
@@ -1341,7 +1341,7 @@
         <v>128</v>
       </c>
       <c r="C29">
-        <v>0.1517371</v>
+        <v>0.1549465</v>
       </c>
       <c r="D29" t="s">
         <v>3</v>
@@ -1353,7 +1353,7 @@
         <v>203.0365799264593</v>
       </c>
       <c r="G29">
-        <v>373</v>
+        <v>387</v>
       </c>
       <c r="H29">
         <v>4034</v>
@@ -1362,7 +1362,7 @@
         <v>20</v>
       </c>
       <c r="J29">
-        <v>4407</v>
+        <v>4421</v>
       </c>
     </row>
     <row r="30" spans="1:10">
@@ -1373,7 +1373,7 @@
         <v>16</v>
       </c>
       <c r="C30">
-        <v>0.0005046</v>
+        <v>0.0004917</v>
       </c>
       <c r="D30" t="s">
         <v>17</v>
@@ -1405,7 +1405,7 @@
         <v>16</v>
       </c>
       <c r="C31">
-        <v>0.0003077</v>
+        <v>0.0002944000000000001</v>
       </c>
       <c r="D31" t="s">
         <v>17</v>
@@ -1437,28 +1437,28 @@
         <v>16</v>
       </c>
       <c r="C32">
-        <v>0.00055</v>
+        <v>0.0002705</v>
       </c>
       <c r="D32" t="s">
         <v>17</v>
       </c>
       <c r="E32">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F32">
-        <v>28.38477631085023</v>
+        <v>25.55634918610405</v>
       </c>
       <c r="G32">
-        <v>39</v>
+        <v>31</v>
       </c>
       <c r="H32">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="I32">
         <v>11</v>
       </c>
       <c r="J32">
-        <v>72</v>
+        <v>63</v>
       </c>
     </row>
     <row r="33" spans="1:10">
@@ -1469,7 +1469,7 @@
         <v>16</v>
       </c>
       <c r="C33">
-        <v>0.0004154</v>
+        <v>0.0004196</v>
       </c>
       <c r="D33" t="s">
         <v>17</v>
@@ -1501,7 +1501,7 @@
         <v>16</v>
       </c>
       <c r="C34">
-        <v>0.0003521</v>
+        <v>0.0004123</v>
       </c>
       <c r="D34" t="s">
         <v>17</v>
@@ -1533,7 +1533,7 @@
         <v>16</v>
       </c>
       <c r="C35">
-        <v>0.0006652</v>
+        <v>0.0004839999999999999</v>
       </c>
       <c r="D35" t="s">
         <v>17</v>
@@ -1542,7 +1542,7 @@
         <v>7</v>
       </c>
       <c r="F35">
-        <v>24.2748964148517</v>
+        <v>24.370154202675</v>
       </c>
       <c r="G35">
         <v>25</v>
@@ -1565,7 +1565,7 @@
         <v>16</v>
       </c>
       <c r="C36">
-        <v>0.0007118000000000001</v>
+        <v>0.0005338</v>
       </c>
       <c r="D36" t="s">
         <v>17</v>
@@ -1577,7 +1577,7 @@
         <v>25.55634918610405</v>
       </c>
       <c r="G36">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="H36">
         <v>69</v>
@@ -1586,7 +1586,7 @@
         <v>12</v>
       </c>
       <c r="J36">
-        <v>93</v>
+        <v>96</v>
       </c>
     </row>
     <row r="37" spans="1:10">
@@ -1597,7 +1597,7 @@
         <v>32</v>
       </c>
       <c r="C37">
-        <v>0.0029849</v>
+        <v>0.0029884</v>
       </c>
       <c r="D37" t="s">
         <v>17</v>
@@ -1629,7 +1629,7 @@
         <v>32</v>
       </c>
       <c r="C38">
-        <v>0.0012901</v>
+        <v>0.00127</v>
       </c>
       <c r="D38" t="s">
         <v>17</v>
@@ -1661,7 +1661,7 @@
         <v>32</v>
       </c>
       <c r="C39">
-        <v>0.0019769</v>
+        <v>0.0009784999999999998</v>
       </c>
       <c r="D39" t="s">
         <v>17</v>
@@ -1670,19 +1670,19 @@
         <v>44</v>
       </c>
       <c r="F39">
-        <v>52.52691193458119</v>
+        <v>51.69848480983499</v>
       </c>
       <c r="G39">
-        <v>105</v>
+        <v>97</v>
       </c>
       <c r="H39">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="I39">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J39">
-        <v>182</v>
+        <v>172</v>
       </c>
     </row>
     <row r="40" spans="1:10">
@@ -1693,7 +1693,7 @@
         <v>32</v>
       </c>
       <c r="C40">
-        <v>0.002414</v>
+        <v>0.002399</v>
       </c>
       <c r="D40" t="s">
         <v>17</v>
@@ -1725,7 +1725,7 @@
         <v>32</v>
       </c>
       <c r="C41">
-        <v>0.0010381</v>
+        <v>0.0010203</v>
       </c>
       <c r="D41" t="s">
         <v>17</v>
@@ -1757,7 +1757,7 @@
         <v>32</v>
       </c>
       <c r="C42">
-        <v>0.0030295</v>
+        <v>0.0029943</v>
       </c>
       <c r="D42" t="s">
         <v>17</v>
@@ -1789,7 +1789,7 @@
         <v>32</v>
       </c>
       <c r="C43">
-        <v>0.0029012</v>
+        <v>0.0028261</v>
       </c>
       <c r="D43" t="s">
         <v>17</v>
@@ -1801,7 +1801,7 @@
         <v>51.69848480983499</v>
       </c>
       <c r="G43">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="H43">
         <v>266</v>
@@ -1810,7 +1810,7 @@
         <v>14</v>
       </c>
       <c r="J43">
-        <v>319</v>
+        <v>322</v>
       </c>
     </row>
     <row r="44" spans="1:10">
@@ -1821,7 +1821,7 @@
         <v>64</v>
       </c>
       <c r="C44">
-        <v>0.0196066</v>
+        <v>0.0202147</v>
       </c>
       <c r="D44" t="s">
         <v>17</v>
@@ -1853,7 +1853,7 @@
         <v>64</v>
       </c>
       <c r="C45">
-        <v>0.0051455</v>
+        <v>0.0050963</v>
       </c>
       <c r="D45" t="s">
         <v>17</v>
@@ -1885,7 +1885,7 @@
         <v>64</v>
       </c>
       <c r="C46">
-        <v>0.0173749</v>
+        <v>0.005393600000000001</v>
       </c>
       <c r="D46" t="s">
         <v>17</v>
@@ -1894,19 +1894,19 @@
         <v>88</v>
       </c>
       <c r="F46">
-        <v>107.2964645562817</v>
+        <v>104.8111831820431</v>
       </c>
       <c r="G46">
-        <v>331</v>
+        <v>252</v>
       </c>
       <c r="H46">
-        <v>395</v>
+        <v>229</v>
       </c>
       <c r="I46">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J46">
-        <v>726</v>
+        <v>481</v>
       </c>
     </row>
     <row r="47" spans="1:10">
@@ -1917,7 +1917,7 @@
         <v>64</v>
       </c>
       <c r="C47">
-        <v>0.0163651</v>
+        <v>0.0166019</v>
       </c>
       <c r="D47" t="s">
         <v>17</v>
@@ -1949,7 +1949,7 @@
         <v>64</v>
       </c>
       <c r="C48">
-        <v>0.0034979</v>
+        <v>0.0035396</v>
       </c>
       <c r="D48" t="s">
         <v>17</v>
@@ -1981,7 +1981,7 @@
         <v>64</v>
       </c>
       <c r="C49">
-        <v>0.0197748</v>
+        <v>0.0199947</v>
       </c>
       <c r="D49" t="s">
         <v>17</v>
@@ -2013,7 +2013,7 @@
         <v>64</v>
       </c>
       <c r="C50">
-        <v>0.0183939</v>
+        <v>0.0189401</v>
       </c>
       <c r="D50" t="s">
         <v>17</v>
@@ -2045,7 +2045,7 @@
         <v>128</v>
       </c>
       <c r="C51">
-        <v>0.1302875</v>
+        <v>0.1326106</v>
       </c>
       <c r="D51" t="s">
         <v>17</v>
@@ -2077,7 +2077,7 @@
         <v>128</v>
       </c>
       <c r="C52">
-        <v>0.0220098</v>
+        <v>0.0216924</v>
       </c>
       <c r="D52" t="s">
         <v>17</v>
@@ -2109,7 +2109,7 @@
         <v>128</v>
       </c>
       <c r="C53">
-        <v>0.1626759</v>
+        <v>0.0299984</v>
       </c>
       <c r="D53" t="s">
         <v>17</v>
@@ -2118,19 +2118,19 @@
         <v>176</v>
       </c>
       <c r="F53">
-        <v>214.350288425444</v>
+        <v>211.8650070512055</v>
       </c>
       <c r="G53">
-        <v>836</v>
+        <v>540</v>
       </c>
       <c r="H53">
-        <v>1847</v>
+        <v>735</v>
       </c>
       <c r="I53">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="J53">
-        <v>2683</v>
+        <v>1275</v>
       </c>
     </row>
     <row r="54" spans="1:10">
@@ -2141,7 +2141,7 @@
         <v>128</v>
       </c>
       <c r="C54">
-        <v>0.1147033</v>
+        <v>0.1168257</v>
       </c>
       <c r="D54" t="s">
         <v>17</v>
@@ -2173,7 +2173,7 @@
         <v>128</v>
       </c>
       <c r="C55">
-        <v>0.0127862</v>
+        <v>0.0133145</v>
       </c>
       <c r="D55" t="s">
         <v>17</v>
@@ -2205,7 +2205,7 @@
         <v>128</v>
       </c>
       <c r="C56">
-        <v>0.1311289</v>
+        <v>0.1322051</v>
       </c>
       <c r="D56" t="s">
         <v>17</v>
@@ -2237,7 +2237,7 @@
         <v>128</v>
       </c>
       <c r="C57">
-        <v>0.1253862</v>
+        <v>0.1285134</v>
       </c>
       <c r="D57" t="s">
         <v>17</v>
@@ -2249,7 +2249,7 @@
         <v>208.5512985522207</v>
       </c>
       <c r="G57">
-        <v>322</v>
+        <v>336</v>
       </c>
       <c r="H57">
         <v>4201</v>
@@ -2258,7 +2258,7 @@
         <v>24</v>
       </c>
       <c r="J57">
-        <v>4523</v>
+        <v>4537</v>
       </c>
     </row>
     <row r="58" spans="1:10">
@@ -2269,7 +2269,7 @@
         <v>16</v>
       </c>
       <c r="C58">
-        <v>0.000411</v>
+        <v>0.0003857</v>
       </c>
       <c r="D58" t="s">
         <v>18</v>
@@ -2301,7 +2301,7 @@
         <v>16</v>
       </c>
       <c r="C59">
-        <v>0.000229</v>
+        <v>0.0002344</v>
       </c>
       <c r="D59" t="s">
         <v>18</v>
@@ -2333,28 +2333,28 @@
         <v>16</v>
       </c>
       <c r="C60">
-        <v>0.0003135</v>
+        <v>0.0001989</v>
       </c>
       <c r="D60" t="s">
         <v>18</v>
       </c>
       <c r="E60">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F60">
-        <v>26.72792206135786</v>
+        <v>25.31370849898476</v>
       </c>
       <c r="G60">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="H60">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="I60">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="J60">
-        <v>44</v>
+        <v>51</v>
       </c>
     </row>
     <row r="61" spans="1:10">
@@ -2365,7 +2365,7 @@
         <v>16</v>
       </c>
       <c r="C61">
-        <v>0.0003295</v>
+        <v>0.0003264</v>
       </c>
       <c r="D61" t="s">
         <v>18</v>
@@ -2397,7 +2397,7 @@
         <v>16</v>
       </c>
       <c r="C62">
-        <v>0.0004089</v>
+        <v>0.0004107000000000001</v>
       </c>
       <c r="D62" t="s">
         <v>18</v>
@@ -2429,16 +2429,16 @@
         <v>16</v>
       </c>
       <c r="C63">
-        <v>0.0004338</v>
+        <v>0.0003958</v>
       </c>
       <c r="D63" t="s">
         <v>18</v>
       </c>
       <c r="E63">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F63">
-        <v>24.32285268768197</v>
+        <v>24.54572853696417</v>
       </c>
       <c r="G63">
         <v>13</v>
@@ -2447,7 +2447,7 @@
         <v>59</v>
       </c>
       <c r="I63">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="J63">
         <v>72</v>
@@ -2461,7 +2461,7 @@
         <v>16</v>
       </c>
       <c r="C64">
-        <v>0.0004282</v>
+        <v>0.0004186</v>
       </c>
       <c r="D64" t="s">
         <v>18</v>
@@ -2473,7 +2473,7 @@
         <v>25.31370849898476</v>
       </c>
       <c r="G64">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H64">
         <v>62</v>
@@ -2482,7 +2482,7 @@
         <v>13</v>
       </c>
       <c r="J64">
-        <v>76</v>
+        <v>77</v>
       </c>
     </row>
     <row r="65" spans="1:10">
@@ -2493,7 +2493,7 @@
         <v>32</v>
       </c>
       <c r="C65">
-        <v>0.0025615</v>
+        <v>0.0025202</v>
       </c>
       <c r="D65" t="s">
         <v>18</v>
@@ -2525,7 +2525,7 @@
         <v>32</v>
       </c>
       <c r="C66">
-        <v>0.0010567</v>
+        <v>0.0010261</v>
       </c>
       <c r="D66" t="s">
         <v>18</v>
@@ -2557,7 +2557,7 @@
         <v>32</v>
       </c>
       <c r="C67">
-        <v>0.0014422</v>
+        <v>0.0007438999999999999</v>
       </c>
       <c r="D67" t="s">
         <v>18</v>
@@ -2569,16 +2569,16 @@
         <v>54.04163056034262</v>
       </c>
       <c r="G67">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="H67">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="I67">
         <v>16</v>
       </c>
       <c r="J67">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="68" spans="1:10">
@@ -2589,7 +2589,7 @@
         <v>32</v>
       </c>
       <c r="C68">
-        <v>0.0020269</v>
+        <v>0.0019956</v>
       </c>
       <c r="D68" t="s">
         <v>18</v>
@@ -2621,7 +2621,7 @@
         <v>32</v>
       </c>
       <c r="C69">
-        <v>0.0013142</v>
+        <v>0.0013024</v>
       </c>
       <c r="D69" t="s">
         <v>18</v>
@@ -2653,7 +2653,7 @@
         <v>32</v>
       </c>
       <c r="C70">
-        <v>0.002598899999999999</v>
+        <v>0.0025725</v>
       </c>
       <c r="D70" t="s">
         <v>18</v>
@@ -2685,7 +2685,7 @@
         <v>32</v>
       </c>
       <c r="C71">
-        <v>0.0024118</v>
+        <v>0.0023666</v>
       </c>
       <c r="D71" t="s">
         <v>18</v>
@@ -2697,7 +2697,7 @@
         <v>52.04163056034262</v>
       </c>
       <c r="G71">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="H71">
         <v>248</v>
@@ -2706,7 +2706,7 @@
         <v>12</v>
       </c>
       <c r="J71">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="72" spans="1:10">
@@ -2717,7 +2717,7 @@
         <v>64</v>
       </c>
       <c r="C72">
-        <v>0.0168613</v>
+        <v>0.0171838</v>
       </c>
       <c r="D72" t="s">
         <v>18</v>
@@ -2749,7 +2749,7 @@
         <v>64</v>
       </c>
       <c r="C73">
-        <v>0.004311999999999999</v>
+        <v>0.0043424</v>
       </c>
       <c r="D73" t="s">
         <v>18</v>
@@ -2781,28 +2781,28 @@
         <v>64</v>
       </c>
       <c r="C74">
-        <v>0.0093718</v>
+        <v>0.002988</v>
       </c>
       <c r="D74" t="s">
         <v>18</v>
       </c>
       <c r="E74">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="F74">
-        <v>106.3259018078045</v>
+        <v>108.6690475583121</v>
       </c>
       <c r="G74">
-        <v>229</v>
+        <v>174</v>
       </c>
       <c r="H74">
-        <v>267</v>
+        <v>144</v>
       </c>
       <c r="I74">
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="J74">
-        <v>496</v>
+        <v>318</v>
       </c>
     </row>
     <row r="75" spans="1:10">
@@ -2813,7 +2813,7 @@
         <v>64</v>
       </c>
       <c r="C75">
-        <v>0.0135943</v>
+        <v>0.0142777</v>
       </c>
       <c r="D75" t="s">
         <v>18</v>
@@ -2845,7 +2845,7 @@
         <v>64</v>
       </c>
       <c r="C76">
-        <v>0.004973300000000001</v>
+        <v>0.004972600000000001</v>
       </c>
       <c r="D76" t="s">
         <v>18</v>
@@ -2877,7 +2877,7 @@
         <v>64</v>
       </c>
       <c r="C77">
-        <v>0.0171851</v>
+        <v>0.0173022</v>
       </c>
       <c r="D77" t="s">
         <v>18</v>
@@ -2909,7 +2909,7 @@
         <v>64</v>
       </c>
       <c r="C78">
-        <v>0.0149212</v>
+        <v>0.0151008</v>
       </c>
       <c r="D78" t="s">
         <v>18</v>
@@ -2921,7 +2921,7 @@
         <v>105.4974746830583</v>
       </c>
       <c r="G78">
-        <v>104</v>
+        <v>108</v>
       </c>
       <c r="H78">
         <v>995</v>
@@ -2930,7 +2930,7 @@
         <v>18</v>
       </c>
       <c r="J78">
-        <v>1099</v>
+        <v>1103</v>
       </c>
     </row>
     <row r="79" spans="1:10">
@@ -2941,7 +2941,7 @@
         <v>128</v>
       </c>
       <c r="C79">
-        <v>0.1104541</v>
+        <v>0.1113246</v>
       </c>
       <c r="D79" t="s">
         <v>18</v>
@@ -2973,7 +2973,7 @@
         <v>128</v>
       </c>
       <c r="C80">
-        <v>0.0179439</v>
+        <v>0.0178264</v>
       </c>
       <c r="D80" t="s">
         <v>18</v>
@@ -3005,28 +3005,28 @@
         <v>128</v>
       </c>
       <c r="C81">
-        <v>0.07056939999999999</v>
+        <v>0.0138025</v>
       </c>
       <c r="D81" t="s">
         <v>18</v>
       </c>
       <c r="E81">
-        <v>184</v>
+        <v>192</v>
       </c>
       <c r="F81">
-        <v>214.0660171779821</v>
+        <v>218.7523086789974</v>
       </c>
       <c r="G81">
-        <v>544</v>
+        <v>417</v>
       </c>
       <c r="H81">
-        <v>1070</v>
+        <v>394</v>
       </c>
       <c r="I81">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="J81">
-        <v>1614</v>
+        <v>811</v>
       </c>
     </row>
     <row r="82" spans="1:10">
@@ -3037,7 +3037,7 @@
         <v>128</v>
       </c>
       <c r="C82">
-        <v>0.08971359999999999</v>
+        <v>0.09037300000000001</v>
       </c>
       <c r="D82" t="s">
         <v>18</v>
@@ -3069,7 +3069,7 @@
         <v>128</v>
       </c>
       <c r="C83">
-        <v>0.0216076</v>
+        <v>0.0217999</v>
       </c>
       <c r="D83" t="s">
         <v>18</v>
@@ -3101,7 +3101,7 @@
         <v>128</v>
       </c>
       <c r="C84">
-        <v>0.1110167</v>
+        <v>0.1117027</v>
       </c>
       <c r="D84" t="s">
         <v>18</v>
@@ -3133,7 +3133,7 @@
         <v>128</v>
       </c>
       <c r="C85">
-        <v>0.0993503</v>
+        <v>0.1007172</v>
       </c>
       <c r="D85" t="s">
         <v>18</v>
@@ -3145,7 +3145,7 @@
         <v>212.4091629284898</v>
       </c>
       <c r="G85">
-        <v>247</v>
+        <v>248</v>
       </c>
       <c r="H85">
         <v>3952</v>
@@ -3154,7 +3154,7 @@
         <v>20</v>
       </c>
       <c r="J85">
-        <v>4199</v>
+        <v>4200</v>
       </c>
     </row>
     <row r="86" spans="1:10">
@@ -3165,7 +3165,7 @@
         <v>16</v>
       </c>
       <c r="C86">
-        <v>0.0006736</v>
+        <v>0.0005730000000000001</v>
       </c>
       <c r="D86" t="s">
         <v>19</v>
@@ -3197,7 +3197,7 @@
         <v>16</v>
       </c>
       <c r="C87">
-        <v>0.00026</v>
+        <v>0.0002544</v>
       </c>
       <c r="D87" t="s">
         <v>19</v>
@@ -3229,7 +3229,7 @@
         <v>16</v>
       </c>
       <c r="C88">
-        <v>0.0003932000000000001</v>
+        <v>0.000196</v>
       </c>
       <c r="D88" t="s">
         <v>19</v>
@@ -3261,7 +3261,7 @@
         <v>16</v>
       </c>
       <c r="C89">
-        <v>0.000454</v>
+        <v>0.0004541000000000001</v>
       </c>
       <c r="D89" t="s">
         <v>19</v>
@@ -3293,7 +3293,7 @@
         <v>16</v>
       </c>
       <c r="C90">
-        <v>0.0004305</v>
+        <v>0.0004201</v>
       </c>
       <c r="D90" t="s">
         <v>19</v>
@@ -3325,7 +3325,7 @@
         <v>16</v>
       </c>
       <c r="C91">
-        <v>0.0007059999999999999</v>
+        <v>0.0005912000000000001</v>
       </c>
       <c r="D91" t="s">
         <v>19</v>
@@ -3334,7 +3334,7 @@
         <v>6</v>
       </c>
       <c r="F91">
-        <v>22.56073125075471</v>
+        <v>22.73887683562801</v>
       </c>
       <c r="G91">
         <v>34</v>
@@ -3357,7 +3357,7 @@
         <v>16</v>
       </c>
       <c r="C92">
-        <v>0.0006441000000000001</v>
+        <v>0.0005688000000000001</v>
       </c>
       <c r="D92" t="s">
         <v>19</v>
@@ -3369,10 +3369,10 @@
         <v>23.55634918610405</v>
       </c>
       <c r="G92">
-        <v>35</v>
+        <v>38</v>
       </c>
       <c r="H92">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="I92">
         <v>11</v>
@@ -3389,7 +3389,7 @@
         <v>32</v>
       </c>
       <c r="C93">
-        <v>0.003875100000000001</v>
+        <v>0.0039611</v>
       </c>
       <c r="D93" t="s">
         <v>19</v>
@@ -3421,7 +3421,7 @@
         <v>32</v>
       </c>
       <c r="C94">
-        <v>0.0011789</v>
+        <v>0.0011466</v>
       </c>
       <c r="D94" t="s">
         <v>19</v>
@@ -3453,7 +3453,7 @@
         <v>32</v>
       </c>
       <c r="C95">
-        <v>0.0014195</v>
+        <v>0.0006352</v>
       </c>
       <c r="D95" t="s">
         <v>19</v>
@@ -3462,19 +3462,19 @@
         <v>40</v>
       </c>
       <c r="F95">
-        <v>50.18376618407358</v>
+        <v>49.35533905932738</v>
       </c>
       <c r="G95">
         <v>91</v>
       </c>
       <c r="H95">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="I95">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="J95">
-        <v>152</v>
+        <v>140</v>
       </c>
     </row>
     <row r="96" spans="1:10">
@@ -3485,7 +3485,7 @@
         <v>32</v>
       </c>
       <c r="C96">
-        <v>0.002692</v>
+        <v>0.0026946</v>
       </c>
       <c r="D96" t="s">
         <v>19</v>
@@ -3517,7 +3517,7 @@
         <v>32</v>
       </c>
       <c r="C97">
-        <v>0.0013392</v>
+        <v>0.0013573</v>
       </c>
       <c r="D97" t="s">
         <v>19</v>
@@ -3549,7 +3549,7 @@
         <v>32</v>
       </c>
       <c r="C98">
-        <v>0.0039451</v>
+        <v>0.0038404</v>
       </c>
       <c r="D98" t="s">
         <v>19</v>
@@ -3581,7 +3581,7 @@
         <v>32</v>
       </c>
       <c r="C99">
-        <v>0.0044204</v>
+        <v>0.0037471</v>
       </c>
       <c r="D99" t="s">
         <v>19</v>
@@ -3593,7 +3593,7 @@
         <v>48.52691193458118</v>
       </c>
       <c r="G99">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="H99">
         <v>289</v>
@@ -3602,7 +3602,7 @@
         <v>12</v>
       </c>
       <c r="J99">
-        <v>377</v>
+        <v>382</v>
       </c>
     </row>
     <row r="100" spans="1:10">
@@ -3613,7 +3613,7 @@
         <v>64</v>
       </c>
       <c r="C100">
-        <v>0.0296328</v>
+        <v>0.0298233</v>
       </c>
       <c r="D100" t="s">
         <v>19</v>
@@ -3645,7 +3645,7 @@
         <v>64</v>
       </c>
       <c r="C101">
-        <v>0.0051299</v>
+        <v>0.0050745</v>
       </c>
       <c r="D101" t="s">
         <v>19</v>
@@ -3677,28 +3677,28 @@
         <v>64</v>
       </c>
       <c r="C102">
-        <v>0.0058033</v>
+        <v>0.0026319</v>
       </c>
       <c r="D102" t="s">
         <v>19</v>
       </c>
       <c r="E102">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="F102">
-        <v>102.3675323681472</v>
+        <v>100.953318805774</v>
       </c>
       <c r="G102">
-        <v>230</v>
+        <v>216</v>
       </c>
       <c r="H102">
-        <v>160</v>
+        <v>115</v>
       </c>
       <c r="I102">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="J102">
-        <v>390</v>
+        <v>331</v>
       </c>
     </row>
     <row r="103" spans="1:10">
@@ -3709,7 +3709,7 @@
         <v>64</v>
       </c>
       <c r="C103">
-        <v>0.0183267</v>
+        <v>0.0186878</v>
       </c>
       <c r="D103" t="s">
         <v>19</v>
@@ -3741,7 +3741,7 @@
         <v>64</v>
       </c>
       <c r="C104">
-        <v>0.0050223</v>
+        <v>0.0050461</v>
       </c>
       <c r="D104" t="s">
         <v>19</v>
@@ -3773,7 +3773,7 @@
         <v>64</v>
       </c>
       <c r="C105">
-        <v>0.029346</v>
+        <v>0.0296411</v>
       </c>
       <c r="D105" t="s">
         <v>19</v>
@@ -3805,7 +3805,7 @@
         <v>64</v>
       </c>
       <c r="C106">
-        <v>0.0279673</v>
+        <v>0.028635</v>
       </c>
       <c r="D106" t="s">
         <v>19</v>
@@ -3817,7 +3817,7 @@
         <v>98.46803743153546</v>
       </c>
       <c r="G106">
-        <v>286</v>
+        <v>297</v>
       </c>
       <c r="H106">
         <v>1212</v>
@@ -3826,7 +3826,7 @@
         <v>12</v>
       </c>
       <c r="J106">
-        <v>1498</v>
+        <v>1509</v>
       </c>
     </row>
     <row r="107" spans="1:10">
@@ -3837,7 +3837,7 @@
         <v>128</v>
       </c>
       <c r="C107">
-        <v>0.2242598</v>
+        <v>0.2253527</v>
       </c>
       <c r="D107" t="s">
         <v>19</v>
@@ -3869,7 +3869,7 @@
         <v>128</v>
       </c>
       <c r="C108">
-        <v>0.022055</v>
+        <v>0.0216949</v>
       </c>
       <c r="D108" t="s">
         <v>19</v>
@@ -3901,28 +3901,28 @@
         <v>128</v>
       </c>
       <c r="C109">
-        <v>0.0368362</v>
+        <v>0.0129174</v>
       </c>
       <c r="D109" t="s">
         <v>19</v>
       </c>
       <c r="E109">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F109">
-        <v>204.7350647362943</v>
+        <v>203.3208511739212</v>
       </c>
       <c r="G109">
-        <v>625</v>
+        <v>488</v>
       </c>
       <c r="H109">
-        <v>581</v>
+        <v>316</v>
       </c>
       <c r="I109">
-        <v>29</v>
+        <v>21</v>
       </c>
       <c r="J109">
-        <v>1206</v>
+        <v>804</v>
       </c>
     </row>
     <row r="110" spans="1:10">
@@ -3933,7 +3933,7 @@
         <v>128</v>
       </c>
       <c r="C110">
-        <v>0.1254835</v>
+        <v>0.1292262</v>
       </c>
       <c r="D110" t="s">
         <v>19</v>
@@ -3965,7 +3965,7 @@
         <v>128</v>
       </c>
       <c r="C111">
-        <v>0.0206832</v>
+        <v>0.020667</v>
       </c>
       <c r="D111" t="s">
         <v>19</v>
@@ -3997,7 +3997,7 @@
         <v>128</v>
       </c>
       <c r="C112">
-        <v>0.2232106</v>
+        <v>0.2263918</v>
       </c>
       <c r="D112" t="s">
         <v>19</v>
@@ -4029,7 +4029,7 @@
         <v>128</v>
       </c>
       <c r="C113">
-        <v>0.2098544</v>
+        <v>0.2141135</v>
       </c>
       <c r="D113" t="s">
         <v>19</v>
@@ -4041,7 +4041,7 @@
         <v>198.350288425444</v>
       </c>
       <c r="G113">
-        <v>706</v>
+        <v>744</v>
       </c>
       <c r="H113">
         <v>4951</v>
@@ -4050,7 +4050,7 @@
         <v>18</v>
       </c>
       <c r="J113">
-        <v>5657</v>
+        <v>5695</v>
       </c>
     </row>
     <row r="114" spans="1:10">
@@ -4061,7 +4061,7 @@
         <v>16</v>
       </c>
       <c r="C114">
-        <v>0.0007793</v>
+        <v>0.0014131</v>
       </c>
       <c r="D114" t="s">
         <v>20</v>
@@ -4093,7 +4093,7 @@
         <v>16</v>
       </c>
       <c r="C115">
-        <v>0.00029</v>
+        <v>0.000253</v>
       </c>
       <c r="D115" t="s">
         <v>20</v>
@@ -4125,7 +4125,7 @@
         <v>16</v>
       </c>
       <c r="C116">
-        <v>0.0004352</v>
+        <v>0.0001992</v>
       </c>
       <c r="D116" t="s">
         <v>20</v>
@@ -4137,10 +4137,10 @@
         <v>24.38477631085024</v>
       </c>
       <c r="G116">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="H116">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="I116">
         <v>7</v>
@@ -4157,7 +4157,7 @@
         <v>16</v>
       </c>
       <c r="C117">
-        <v>0.0006098</v>
+        <v>0.0006092999999999999</v>
       </c>
       <c r="D117" t="s">
         <v>20</v>
@@ -4189,7 +4189,7 @@
         <v>16</v>
       </c>
       <c r="C118">
-        <v>0.0006093</v>
+        <v>0.0006078</v>
       </c>
       <c r="D118" t="s">
         <v>20</v>
@@ -4221,7 +4221,7 @@
         <v>16</v>
       </c>
       <c r="C119">
-        <v>0.0008636999999999999</v>
+        <v>0.0008003999999999999</v>
       </c>
       <c r="D119" t="s">
         <v>20</v>
@@ -4253,7 +4253,7 @@
         <v>16</v>
       </c>
       <c r="C120">
-        <v>0.0009927</v>
+        <v>0.0010103</v>
       </c>
       <c r="D120" t="s">
         <v>20</v>
@@ -4285,7 +4285,7 @@
         <v>32</v>
       </c>
       <c r="C121">
-        <v>0.0057743</v>
+        <v>0.005987899999999999</v>
       </c>
       <c r="D121" t="s">
         <v>20</v>
@@ -4317,7 +4317,7 @@
         <v>32</v>
       </c>
       <c r="C122">
-        <v>0.0009507</v>
+        <v>0.0009589000000000001</v>
       </c>
       <c r="D122" t="s">
         <v>20</v>
@@ -4349,7 +4349,7 @@
         <v>32</v>
       </c>
       <c r="C123">
-        <v>0.0015813</v>
+        <v>0.0005905999999999999</v>
       </c>
       <c r="D123" t="s">
         <v>20</v>
@@ -4361,16 +4361,16 @@
         <v>49.35533905932738</v>
       </c>
       <c r="G123">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="H123">
-        <v>58</v>
+        <v>40</v>
       </c>
       <c r="I123">
         <v>8</v>
       </c>
       <c r="J123">
-        <v>162</v>
+        <v>142</v>
       </c>
     </row>
     <row r="124" spans="1:10">
@@ -4381,7 +4381,7 @@
         <v>32</v>
       </c>
       <c r="C124">
-        <v>0.0035952</v>
+        <v>0.003592799999999999</v>
       </c>
       <c r="D124" t="s">
         <v>20</v>
@@ -4413,7 +4413,7 @@
         <v>32</v>
       </c>
       <c r="C125">
-        <v>0.0021138</v>
+        <v>0.0021167</v>
       </c>
       <c r="D125" t="s">
         <v>20</v>
@@ -4445,7 +4445,7 @@
         <v>32</v>
       </c>
       <c r="C126">
-        <v>0.0058417</v>
+        <v>0.0058376</v>
       </c>
       <c r="D126" t="s">
         <v>20</v>
@@ -4477,7 +4477,7 @@
         <v>32</v>
       </c>
       <c r="C127">
-        <v>0.007036299999999998</v>
+        <v>0.0069051</v>
       </c>
       <c r="D127" t="s">
         <v>20</v>
@@ -4489,7 +4489,7 @@
         <v>47.35533905932738</v>
       </c>
       <c r="G127">
-        <v>214</v>
+        <v>230</v>
       </c>
       <c r="H127">
         <v>337</v>
@@ -4498,7 +4498,7 @@
         <v>8</v>
       </c>
       <c r="J127">
-        <v>551</v>
+        <v>567</v>
       </c>
     </row>
     <row r="128" spans="1:10">
@@ -4509,7 +4509,7 @@
         <v>64</v>
       </c>
       <c r="C128">
-        <v>0.0501117</v>
+        <v>0.0491155</v>
       </c>
       <c r="D128" t="s">
         <v>20</v>
@@ -4541,7 +4541,7 @@
         <v>64</v>
       </c>
       <c r="C129">
-        <v>0.0037831</v>
+        <v>0.003908</v>
       </c>
       <c r="D129" t="s">
         <v>20</v>
@@ -4573,7 +4573,7 @@
         <v>64</v>
       </c>
       <c r="C130">
-        <v>0.0118541</v>
+        <v>0.0020338</v>
       </c>
       <c r="D130" t="s">
         <v>20</v>
@@ -4585,16 +4585,16 @@
         <v>100.1248916810278</v>
       </c>
       <c r="G130">
-        <v>292</v>
+        <v>223</v>
       </c>
       <c r="H130">
-        <v>263</v>
+        <v>85</v>
       </c>
       <c r="I130">
         <v>8</v>
       </c>
       <c r="J130">
-        <v>555</v>
+        <v>308</v>
       </c>
     </row>
     <row r="131" spans="1:10">
@@ -4605,7 +4605,7 @@
         <v>64</v>
       </c>
       <c r="C131">
-        <v>0.023993</v>
+        <v>0.0239114</v>
       </c>
       <c r="D131" t="s">
         <v>20</v>
@@ -4637,7 +4637,7 @@
         <v>64</v>
       </c>
       <c r="C132">
-        <v>0.0080479</v>
+        <v>0.008017800000000002</v>
       </c>
       <c r="D132" t="s">
         <v>20</v>
@@ -4669,7 +4669,7 @@
         <v>64</v>
       </c>
       <c r="C133">
-        <v>0.0502154</v>
+        <v>0.0494466</v>
       </c>
       <c r="D133" t="s">
         <v>20</v>
@@ -4701,7 +4701,7 @@
         <v>64</v>
       </c>
       <c r="C134">
-        <v>0.0504695</v>
+        <v>0.0511769</v>
       </c>
       <c r="D134" t="s">
         <v>20</v>
@@ -4713,7 +4713,7 @@
         <v>96.12489168102785</v>
       </c>
       <c r="G134">
-        <v>503</v>
+        <v>526</v>
       </c>
       <c r="H134">
         <v>1301</v>
@@ -4722,7 +4722,7 @@
         <v>14</v>
       </c>
       <c r="J134">
-        <v>1804</v>
+        <v>1827</v>
       </c>
     </row>
     <row r="135" spans="1:10">
@@ -4733,7 +4733,7 @@
         <v>128</v>
       </c>
       <c r="C135">
-        <v>0.340181</v>
+        <v>0.3437210000000001</v>
       </c>
       <c r="D135" t="s">
         <v>20</v>
@@ -4765,7 +4765,7 @@
         <v>128</v>
       </c>
       <c r="C136">
-        <v>0.0173789</v>
+        <v>0.0157092</v>
       </c>
       <c r="D136" t="s">
         <v>20</v>
@@ -4797,28 +4797,28 @@
         <v>128</v>
       </c>
       <c r="C137">
-        <v>0.09822610000000001</v>
+        <v>0.0075347</v>
       </c>
       <c r="D137" t="s">
         <v>20</v>
       </c>
       <c r="E137">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F137">
-        <v>202.2497833620557</v>
+        <v>201.6639969244288</v>
       </c>
       <c r="G137">
-        <v>614</v>
+        <v>476</v>
       </c>
       <c r="H137">
-        <v>1176</v>
+        <v>188</v>
       </c>
       <c r="I137">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J137">
-        <v>1790</v>
+        <v>664</v>
       </c>
     </row>
     <row r="138" spans="1:10">
@@ -4829,7 +4829,7 @@
         <v>128</v>
       </c>
       <c r="C138">
-        <v>0.1622748</v>
+        <v>0.1644629</v>
       </c>
       <c r="D138" t="s">
         <v>20</v>
@@ -4861,7 +4861,7 @@
         <v>128</v>
       </c>
       <c r="C139">
-        <v>0.03305300000000001</v>
+        <v>0.0331036</v>
       </c>
       <c r="D139" t="s">
         <v>20</v>
@@ -4893,7 +4893,7 @@
         <v>128</v>
       </c>
       <c r="C140">
-        <v>0.3422766</v>
+        <v>0.3435911</v>
       </c>
       <c r="D140" t="s">
         <v>20</v>
@@ -4925,7 +4925,7 @@
         <v>128</v>
       </c>
       <c r="C141">
-        <v>0.3391801</v>
+        <v>0.3472421</v>
       </c>
       <c r="D141" t="s">
         <v>20</v>
@@ -4937,7 +4937,7 @@
         <v>193.6639969244288</v>
       </c>
       <c r="G141">
-        <v>1042</v>
+        <v>1079</v>
       </c>
       <c r="H141">
         <v>5069</v>
@@ -4946,7 +4946,7 @@
         <v>22</v>
       </c>
       <c r="J141">
-        <v>6111</v>
+        <v>6148</v>
       </c>
     </row>
   </sheetData>

</xml_diff>